<commit_message>
Implementación inicial del nuevo MVC al estilo Laravel.
</commit_message>
<xml_diff>
--- a/documentacion/ACTAS PONDERADAS BASICO -2021.xlsx
+++ b/documentacion/ACTAS PONDERADAS BASICO -2021.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN-MINEDUC\Desktop\año lectivo 2021 2022\calificaciones 2021\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\rubrica\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="10215" windowHeight="7830"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="10212" windowHeight="7836"/>
   </bookViews>
   <sheets>
     <sheet name="P1" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
     <sheet name="PE" sheetId="4" r:id="rId3"/>
     <sheet name="QUIMESTRE 1" sheetId="3" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -262,7 +262,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -451,15 +451,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -472,16 +463,25 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -527,7 +527,7 @@
         <xdr:cNvPr id="2" name="Imagen 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -582,7 +582,7 @@
         <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0100-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -637,7 +637,7 @@
         <xdr:cNvPr id="2" name="Imagen 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{330DDC9A-4835-4100-9A3E-3E0E73BDB072}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{330DDC9A-4835-4100-9A3E-3E0E73BDB072}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -692,7 +692,7 @@
         <xdr:cNvPr id="4" name="Imagen 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0200-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -991,395 +991,395 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AQ30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.140625" customWidth="1"/>
-    <col min="2" max="2" width="44.42578125" customWidth="1"/>
-    <col min="3" max="3" width="5.85546875" customWidth="1"/>
-    <col min="4" max="4" width="7.28515625" customWidth="1"/>
+    <col min="1" max="1" width="4.109375" customWidth="1"/>
+    <col min="2" max="2" width="44.44140625" customWidth="1"/>
+    <col min="3" max="3" width="5.88671875" customWidth="1"/>
+    <col min="4" max="4" width="7.33203125" customWidth="1"/>
     <col min="5" max="5" width="6" customWidth="1"/>
-    <col min="6" max="6" width="0.7109375" customWidth="1"/>
-    <col min="7" max="7" width="6.85546875" customWidth="1"/>
-    <col min="8" max="8" width="7.85546875" customWidth="1"/>
-    <col min="9" max="9" width="7.140625" customWidth="1"/>
-    <col min="10" max="10" width="7.42578125" customWidth="1"/>
-    <col min="11" max="11" width="6.7109375" customWidth="1"/>
-    <col min="12" max="12" width="6.85546875" customWidth="1"/>
-    <col min="13" max="13" width="7.85546875" customWidth="1"/>
-    <col min="14" max="14" width="7.140625" customWidth="1"/>
-    <col min="15" max="15" width="7.42578125" customWidth="1"/>
-    <col min="16" max="16" width="6.7109375" customWidth="1"/>
-    <col min="17" max="17" width="6.85546875" customWidth="1"/>
-    <col min="18" max="18" width="7.85546875" customWidth="1"/>
-    <col min="19" max="19" width="7.140625" customWidth="1"/>
-    <col min="20" max="20" width="7.42578125" customWidth="1"/>
-    <col min="21" max="21" width="6.7109375" customWidth="1"/>
-    <col min="22" max="22" width="6.85546875" customWidth="1"/>
-    <col min="23" max="23" width="7.85546875" customWidth="1"/>
-    <col min="24" max="24" width="7.140625" customWidth="1"/>
-    <col min="25" max="25" width="7.42578125" customWidth="1"/>
-    <col min="26" max="26" width="6.7109375" customWidth="1"/>
-    <col min="27" max="27" width="6.85546875" customWidth="1"/>
-    <col min="28" max="28" width="7.85546875" customWidth="1"/>
-    <col min="29" max="29" width="7.140625" customWidth="1"/>
-    <col min="30" max="30" width="7.42578125" customWidth="1"/>
-    <col min="31" max="31" width="6.7109375" customWidth="1"/>
-    <col min="32" max="32" width="6.85546875" customWidth="1"/>
-    <col min="33" max="33" width="7.85546875" customWidth="1"/>
-    <col min="34" max="34" width="7.140625" customWidth="1"/>
-    <col min="35" max="35" width="7.42578125" customWidth="1"/>
-    <col min="36" max="36" width="6.7109375" customWidth="1"/>
-    <col min="37" max="37" width="6.85546875" customWidth="1"/>
-    <col min="38" max="38" width="7.85546875" customWidth="1"/>
-    <col min="39" max="39" width="7.140625" customWidth="1"/>
-    <col min="40" max="40" width="7.42578125" customWidth="1"/>
-    <col min="41" max="41" width="6.7109375" customWidth="1"/>
-    <col min="42" max="42" width="0.7109375" customWidth="1"/>
+    <col min="6" max="6" width="0.6640625" customWidth="1"/>
+    <col min="7" max="7" width="6.88671875" customWidth="1"/>
+    <col min="8" max="8" width="7.88671875" customWidth="1"/>
+    <col min="9" max="9" width="7.109375" customWidth="1"/>
+    <col min="10" max="10" width="7.44140625" customWidth="1"/>
+    <col min="11" max="11" width="6.6640625" customWidth="1"/>
+    <col min="12" max="12" width="6.88671875" customWidth="1"/>
+    <col min="13" max="13" width="7.88671875" customWidth="1"/>
+    <col min="14" max="14" width="7.109375" customWidth="1"/>
+    <col min="15" max="15" width="7.44140625" customWidth="1"/>
+    <col min="16" max="16" width="6.6640625" customWidth="1"/>
+    <col min="17" max="17" width="6.88671875" customWidth="1"/>
+    <col min="18" max="18" width="7.88671875" customWidth="1"/>
+    <col min="19" max="19" width="7.109375" customWidth="1"/>
+    <col min="20" max="20" width="7.44140625" customWidth="1"/>
+    <col min="21" max="21" width="6.6640625" customWidth="1"/>
+    <col min="22" max="22" width="6.88671875" customWidth="1"/>
+    <col min="23" max="23" width="7.88671875" customWidth="1"/>
+    <col min="24" max="24" width="7.109375" customWidth="1"/>
+    <col min="25" max="25" width="7.44140625" customWidth="1"/>
+    <col min="26" max="26" width="6.6640625" customWidth="1"/>
+    <col min="27" max="27" width="6.88671875" customWidth="1"/>
+    <col min="28" max="28" width="7.88671875" customWidth="1"/>
+    <col min="29" max="29" width="7.109375" customWidth="1"/>
+    <col min="30" max="30" width="7.44140625" customWidth="1"/>
+    <col min="31" max="31" width="6.6640625" customWidth="1"/>
+    <col min="32" max="32" width="6.88671875" customWidth="1"/>
+    <col min="33" max="33" width="7.88671875" customWidth="1"/>
+    <col min="34" max="34" width="7.109375" customWidth="1"/>
+    <col min="35" max="35" width="7.44140625" customWidth="1"/>
+    <col min="36" max="36" width="6.6640625" customWidth="1"/>
+    <col min="37" max="37" width="6.88671875" customWidth="1"/>
+    <col min="38" max="38" width="7.88671875" customWidth="1"/>
+    <col min="39" max="39" width="7.109375" customWidth="1"/>
+    <col min="40" max="40" width="7.44140625" customWidth="1"/>
+    <col min="41" max="41" width="6.6640625" customWidth="1"/>
+    <col min="42" max="42" width="0.6640625" customWidth="1"/>
     <col min="43" max="43" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.25">
-      <c r="A1" s="24"/>
-      <c r="B1" s="24"/>
-      <c r="C1" s="25" t="s">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A1" s="21"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
-      <c r="R1" s="26"/>
-      <c r="S1" s="26"/>
-      <c r="T1" s="26"/>
-      <c r="U1" s="26"/>
-      <c r="V1" s="26"/>
-      <c r="W1" s="26"/>
-      <c r="X1" s="26"/>
-      <c r="Y1" s="26"/>
-      <c r="Z1" s="26"/>
-      <c r="AA1" s="26"/>
-      <c r="AB1" s="26"/>
-      <c r="AC1" s="26"/>
-      <c r="AD1" s="26"/>
-      <c r="AE1" s="26"/>
-      <c r="AF1" s="26"/>
-      <c r="AG1" s="26"/>
-      <c r="AH1" s="26"/>
-      <c r="AI1" s="26"/>
-      <c r="AJ1" s="26"/>
-      <c r="AK1" s="26"/>
-      <c r="AL1" s="26"/>
-      <c r="AM1" s="26"/>
-      <c r="AN1" s="26"/>
-      <c r="AO1" s="26"/>
-      <c r="AP1" s="26"/>
-      <c r="AQ1" s="26"/>
-    </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.25">
-      <c r="A2" s="24"/>
-      <c r="B2" s="24"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
-      <c r="N2" s="26"/>
-      <c r="O2" s="26"/>
-      <c r="P2" s="26"/>
-      <c r="Q2" s="26"/>
-      <c r="R2" s="26"/>
-      <c r="S2" s="26"/>
-      <c r="T2" s="26"/>
-      <c r="U2" s="26"/>
-      <c r="V2" s="26"/>
-      <c r="W2" s="26"/>
-      <c r="X2" s="26"/>
-      <c r="Y2" s="26"/>
-      <c r="Z2" s="26"/>
-      <c r="AA2" s="26"/>
-      <c r="AB2" s="26"/>
-      <c r="AC2" s="26"/>
-      <c r="AD2" s="26"/>
-      <c r="AE2" s="26"/>
-      <c r="AF2" s="26"/>
-      <c r="AG2" s="26"/>
-      <c r="AH2" s="26"/>
-      <c r="AI2" s="26"/>
-      <c r="AJ2" s="26"/>
-      <c r="AK2" s="26"/>
-      <c r="AL2" s="26"/>
-      <c r="AM2" s="26"/>
-      <c r="AN2" s="26"/>
-      <c r="AO2" s="26"/>
-      <c r="AP2" s="26"/>
-      <c r="AQ2" s="26"/>
-    </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.25">
-      <c r="A3" s="24"/>
-      <c r="B3" s="24"/>
-      <c r="C3" s="27" t="s">
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+      <c r="M1" s="23"/>
+      <c r="N1" s="23"/>
+      <c r="O1" s="23"/>
+      <c r="P1" s="23"/>
+      <c r="Q1" s="23"/>
+      <c r="R1" s="23"/>
+      <c r="S1" s="23"/>
+      <c r="T1" s="23"/>
+      <c r="U1" s="23"/>
+      <c r="V1" s="23"/>
+      <c r="W1" s="23"/>
+      <c r="X1" s="23"/>
+      <c r="Y1" s="23"/>
+      <c r="Z1" s="23"/>
+      <c r="AA1" s="23"/>
+      <c r="AB1" s="23"/>
+      <c r="AC1" s="23"/>
+      <c r="AD1" s="23"/>
+      <c r="AE1" s="23"/>
+      <c r="AF1" s="23"/>
+      <c r="AG1" s="23"/>
+      <c r="AH1" s="23"/>
+      <c r="AI1" s="23"/>
+      <c r="AJ1" s="23"/>
+      <c r="AK1" s="23"/>
+      <c r="AL1" s="23"/>
+      <c r="AM1" s="23"/>
+      <c r="AN1" s="23"/>
+      <c r="AO1" s="23"/>
+      <c r="AP1" s="23"/>
+      <c r="AQ1" s="23"/>
+    </row>
+    <row r="2" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A2" s="21"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
+      <c r="P2" s="23"/>
+      <c r="Q2" s="23"/>
+      <c r="R2" s="23"/>
+      <c r="S2" s="23"/>
+      <c r="T2" s="23"/>
+      <c r="U2" s="23"/>
+      <c r="V2" s="23"/>
+      <c r="W2" s="23"/>
+      <c r="X2" s="23"/>
+      <c r="Y2" s="23"/>
+      <c r="Z2" s="23"/>
+      <c r="AA2" s="23"/>
+      <c r="AB2" s="23"/>
+      <c r="AC2" s="23"/>
+      <c r="AD2" s="23"/>
+      <c r="AE2" s="23"/>
+      <c r="AF2" s="23"/>
+      <c r="AG2" s="23"/>
+      <c r="AH2" s="23"/>
+      <c r="AI2" s="23"/>
+      <c r="AJ2" s="23"/>
+      <c r="AK2" s="23"/>
+      <c r="AL2" s="23"/>
+      <c r="AM2" s="23"/>
+      <c r="AN2" s="23"/>
+      <c r="AO2" s="23"/>
+      <c r="AP2" s="23"/>
+      <c r="AQ2" s="23"/>
+    </row>
+    <row r="3" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A3" s="21"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="27"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="27"/>
-      <c r="J3" s="27"/>
-      <c r="K3" s="27"/>
-      <c r="L3" s="27"/>
-      <c r="M3" s="27"/>
-      <c r="N3" s="27"/>
-      <c r="O3" s="27"/>
-      <c r="P3" s="27"/>
-      <c r="Q3" s="27"/>
-      <c r="R3" s="27"/>
-      <c r="S3" s="27"/>
-      <c r="T3" s="27"/>
-      <c r="U3" s="27"/>
-      <c r="V3" s="27"/>
-      <c r="W3" s="28" t="s">
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="24"/>
+      <c r="L3" s="24"/>
+      <c r="M3" s="24"/>
+      <c r="N3" s="24"/>
+      <c r="O3" s="24"/>
+      <c r="P3" s="24"/>
+      <c r="Q3" s="24"/>
+      <c r="R3" s="24"/>
+      <c r="S3" s="24"/>
+      <c r="T3" s="24"/>
+      <c r="U3" s="24"/>
+      <c r="V3" s="24"/>
+      <c r="W3" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="X3" s="29"/>
-      <c r="Y3" s="29"/>
-      <c r="Z3" s="29"/>
-      <c r="AA3" s="29"/>
-      <c r="AB3" s="29"/>
-      <c r="AC3" s="29"/>
-      <c r="AD3" s="29"/>
-      <c r="AE3" s="29"/>
-      <c r="AF3" s="29"/>
-      <c r="AG3" s="29"/>
-      <c r="AH3" s="29"/>
-      <c r="AI3" s="29"/>
-      <c r="AJ3" s="29"/>
-      <c r="AK3" s="29"/>
-      <c r="AL3" s="29"/>
-      <c r="AM3" s="29"/>
-      <c r="AN3" s="29"/>
-      <c r="AO3" s="29"/>
-      <c r="AP3" s="29"/>
-      <c r="AQ3" s="29"/>
-    </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.25">
-      <c r="A4" s="24"/>
-      <c r="B4" s="24"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
-      <c r="K4" s="27"/>
-      <c r="L4" s="27"/>
-      <c r="M4" s="27"/>
-      <c r="N4" s="27"/>
-      <c r="O4" s="27"/>
-      <c r="P4" s="27"/>
-      <c r="Q4" s="27"/>
-      <c r="R4" s="27"/>
-      <c r="S4" s="27"/>
-      <c r="T4" s="27"/>
-      <c r="U4" s="27"/>
-      <c r="V4" s="27"/>
-      <c r="W4" s="29"/>
-      <c r="X4" s="29"/>
-      <c r="Y4" s="29"/>
-      <c r="Z4" s="29"/>
-      <c r="AA4" s="29"/>
-      <c r="AB4" s="29"/>
-      <c r="AC4" s="29"/>
-      <c r="AD4" s="29"/>
-      <c r="AE4" s="29"/>
-      <c r="AF4" s="29"/>
-      <c r="AG4" s="29"/>
-      <c r="AH4" s="29"/>
-      <c r="AI4" s="29"/>
-      <c r="AJ4" s="29"/>
-      <c r="AK4" s="29"/>
-      <c r="AL4" s="29"/>
-      <c r="AM4" s="29"/>
-      <c r="AN4" s="29"/>
-      <c r="AO4" s="29"/>
-      <c r="AP4" s="29"/>
-      <c r="AQ4" s="29"/>
-    </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.25">
-      <c r="A5" s="24"/>
-      <c r="B5" s="24"/>
-      <c r="C5" s="27" t="s">
+      <c r="X3" s="28"/>
+      <c r="Y3" s="28"/>
+      <c r="Z3" s="28"/>
+      <c r="AA3" s="28"/>
+      <c r="AB3" s="28"/>
+      <c r="AC3" s="28"/>
+      <c r="AD3" s="28"/>
+      <c r="AE3" s="28"/>
+      <c r="AF3" s="28"/>
+      <c r="AG3" s="28"/>
+      <c r="AH3" s="28"/>
+      <c r="AI3" s="28"/>
+      <c r="AJ3" s="28"/>
+      <c r="AK3" s="28"/>
+      <c r="AL3" s="28"/>
+      <c r="AM3" s="28"/>
+      <c r="AN3" s="28"/>
+      <c r="AO3" s="28"/>
+      <c r="AP3" s="28"/>
+      <c r="AQ3" s="28"/>
+    </row>
+    <row r="4" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A4" s="21"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
+      <c r="P4" s="24"/>
+      <c r="Q4" s="24"/>
+      <c r="R4" s="24"/>
+      <c r="S4" s="24"/>
+      <c r="T4" s="24"/>
+      <c r="U4" s="24"/>
+      <c r="V4" s="24"/>
+      <c r="W4" s="28"/>
+      <c r="X4" s="28"/>
+      <c r="Y4" s="28"/>
+      <c r="Z4" s="28"/>
+      <c r="AA4" s="28"/>
+      <c r="AB4" s="28"/>
+      <c r="AC4" s="28"/>
+      <c r="AD4" s="28"/>
+      <c r="AE4" s="28"/>
+      <c r="AF4" s="28"/>
+      <c r="AG4" s="28"/>
+      <c r="AH4" s="28"/>
+      <c r="AI4" s="28"/>
+      <c r="AJ4" s="28"/>
+      <c r="AK4" s="28"/>
+      <c r="AL4" s="28"/>
+      <c r="AM4" s="28"/>
+      <c r="AN4" s="28"/>
+      <c r="AO4" s="28"/>
+      <c r="AP4" s="28"/>
+      <c r="AQ4" s="28"/>
+    </row>
+    <row r="5" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A5" s="21"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
-      <c r="K5" s="27"/>
-      <c r="L5" s="27"/>
-      <c r="M5" s="27"/>
-      <c r="N5" s="27"/>
-      <c r="O5" s="27"/>
-      <c r="P5" s="27"/>
-      <c r="Q5" s="27"/>
-      <c r="R5" s="27"/>
-      <c r="S5" s="27"/>
-      <c r="T5" s="27"/>
-      <c r="U5" s="27"/>
-      <c r="V5" s="27"/>
-      <c r="W5" s="29"/>
-      <c r="X5" s="29"/>
-      <c r="Y5" s="29"/>
-      <c r="Z5" s="29"/>
-      <c r="AA5" s="29"/>
-      <c r="AB5" s="29"/>
-      <c r="AC5" s="29"/>
-      <c r="AD5" s="29"/>
-      <c r="AE5" s="29"/>
-      <c r="AF5" s="29"/>
-      <c r="AG5" s="29"/>
-      <c r="AH5" s="29"/>
-      <c r="AI5" s="29"/>
-      <c r="AJ5" s="29"/>
-      <c r="AK5" s="29"/>
-      <c r="AL5" s="29"/>
-      <c r="AM5" s="29"/>
-      <c r="AN5" s="29"/>
-      <c r="AO5" s="29"/>
-      <c r="AP5" s="29"/>
-      <c r="AQ5" s="29"/>
-    </row>
-    <row r="6" spans="1:43" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="24"/>
-      <c r="B6" s="24"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
-      <c r="M6" s="22"/>
-      <c r="N6" s="22"/>
-      <c r="O6" s="22"/>
-      <c r="P6" s="22"/>
-      <c r="Q6" s="22"/>
-      <c r="R6" s="22"/>
-      <c r="S6" s="22"/>
-      <c r="T6" s="22"/>
-      <c r="U6" s="22"/>
-      <c r="V6" s="22"/>
-      <c r="W6" s="22"/>
-      <c r="X6" s="22"/>
-      <c r="Y6" s="22"/>
-      <c r="Z6" s="22"/>
-      <c r="AA6" s="22"/>
-      <c r="AB6" s="22"/>
-      <c r="AC6" s="22"/>
-      <c r="AD6" s="22"/>
-      <c r="AE6" s="22"/>
-      <c r="AF6" s="22"/>
-      <c r="AG6" s="22"/>
-      <c r="AH6" s="22"/>
-      <c r="AI6" s="22"/>
-      <c r="AJ6" s="22"/>
-      <c r="AK6" s="22"/>
-      <c r="AL6" s="22"/>
-      <c r="AM6" s="22"/>
-      <c r="AN6" s="22"/>
-      <c r="AO6" s="22"/>
-      <c r="AP6" s="22"/>
-      <c r="AQ6" s="22"/>
-    </row>
-    <row r="7" spans="1:43" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="24"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="21" t="s">
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="24"/>
+      <c r="M5" s="24"/>
+      <c r="N5" s="24"/>
+      <c r="O5" s="24"/>
+      <c r="P5" s="24"/>
+      <c r="Q5" s="24"/>
+      <c r="R5" s="24"/>
+      <c r="S5" s="24"/>
+      <c r="T5" s="24"/>
+      <c r="U5" s="24"/>
+      <c r="V5" s="24"/>
+      <c r="W5" s="28"/>
+      <c r="X5" s="28"/>
+      <c r="Y5" s="28"/>
+      <c r="Z5" s="28"/>
+      <c r="AA5" s="28"/>
+      <c r="AB5" s="28"/>
+      <c r="AC5" s="28"/>
+      <c r="AD5" s="28"/>
+      <c r="AE5" s="28"/>
+      <c r="AF5" s="28"/>
+      <c r="AG5" s="28"/>
+      <c r="AH5" s="28"/>
+      <c r="AI5" s="28"/>
+      <c r="AJ5" s="28"/>
+      <c r="AK5" s="28"/>
+      <c r="AL5" s="28"/>
+      <c r="AM5" s="28"/>
+      <c r="AN5" s="28"/>
+      <c r="AO5" s="28"/>
+      <c r="AP5" s="28"/>
+      <c r="AQ5" s="28"/>
+    </row>
+    <row r="6" spans="1:43" ht="6.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="21"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="25"/>
+      <c r="J6" s="25"/>
+      <c r="K6" s="25"/>
+      <c r="L6" s="25"/>
+      <c r="M6" s="25"/>
+      <c r="N6" s="25"/>
+      <c r="O6" s="25"/>
+      <c r="P6" s="25"/>
+      <c r="Q6" s="25"/>
+      <c r="R6" s="25"/>
+      <c r="S6" s="25"/>
+      <c r="T6" s="25"/>
+      <c r="U6" s="25"/>
+      <c r="V6" s="25"/>
+      <c r="W6" s="25"/>
+      <c r="X6" s="25"/>
+      <c r="Y6" s="25"/>
+      <c r="Z6" s="25"/>
+      <c r="AA6" s="25"/>
+      <c r="AB6" s="25"/>
+      <c r="AC6" s="25"/>
+      <c r="AD6" s="25"/>
+      <c r="AE6" s="25"/>
+      <c r="AF6" s="25"/>
+      <c r="AG6" s="25"/>
+      <c r="AH6" s="25"/>
+      <c r="AI6" s="25"/>
+      <c r="AJ6" s="25"/>
+      <c r="AK6" s="25"/>
+      <c r="AL6" s="25"/>
+      <c r="AM6" s="25"/>
+      <c r="AN6" s="25"/>
+      <c r="AO6" s="25"/>
+      <c r="AP6" s="25"/>
+      <c r="AQ6" s="25"/>
+    </row>
+    <row r="7" spans="1:43" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="21"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="21" t="s">
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="H7" s="21"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="21" t="s">
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="M7" s="21"/>
-      <c r="N7" s="21"/>
-      <c r="O7" s="21"/>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21" t="s">
+      <c r="M7" s="26"/>
+      <c r="N7" s="26"/>
+      <c r="O7" s="26"/>
+      <c r="P7" s="26"/>
+      <c r="Q7" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="R7" s="21"/>
-      <c r="S7" s="21"/>
-      <c r="T7" s="21"/>
-      <c r="U7" s="21"/>
-      <c r="V7" s="21" t="s">
+      <c r="R7" s="26"/>
+      <c r="S7" s="26"/>
+      <c r="T7" s="26"/>
+      <c r="U7" s="26"/>
+      <c r="V7" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="W7" s="21"/>
-      <c r="X7" s="21"/>
-      <c r="Y7" s="21"/>
-      <c r="Z7" s="21"/>
-      <c r="AA7" s="21" t="s">
+      <c r="W7" s="26"/>
+      <c r="X7" s="26"/>
+      <c r="Y7" s="26"/>
+      <c r="Z7" s="26"/>
+      <c r="AA7" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="AB7" s="21"/>
-      <c r="AC7" s="21"/>
-      <c r="AD7" s="21"/>
-      <c r="AE7" s="21"/>
-      <c r="AF7" s="21" t="s">
+      <c r="AB7" s="26"/>
+      <c r="AC7" s="26"/>
+      <c r="AD7" s="26"/>
+      <c r="AE7" s="26"/>
+      <c r="AF7" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="AG7" s="21"/>
-      <c r="AH7" s="21"/>
-      <c r="AI7" s="21"/>
-      <c r="AJ7" s="21"/>
-      <c r="AK7" s="21" t="s">
+      <c r="AG7" s="26"/>
+      <c r="AH7" s="26"/>
+      <c r="AI7" s="26"/>
+      <c r="AJ7" s="26"/>
+      <c r="AK7" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="AL7" s="21"/>
-      <c r="AM7" s="21"/>
-      <c r="AN7" s="21"/>
-      <c r="AO7" s="21"/>
-      <c r="AP7" s="23" t="s">
+      <c r="AL7" s="26"/>
+      <c r="AM7" s="26"/>
+      <c r="AN7" s="26"/>
+      <c r="AO7" s="26"/>
+      <c r="AP7" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="AQ7" s="23"/>
-    </row>
-    <row r="8" spans="1:43" ht="0.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AQ7" s="29"/>
+    </row>
+    <row r="8" spans="1:43" ht="0.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -1424,7 +1424,7 @@
       <c r="AP8" s="5"/>
       <c r="AQ8" s="5"/>
     </row>
-    <row r="9" spans="1:43" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:43" ht="89.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>0</v>
       </c>
@@ -1440,7 +1440,7 @@
       <c r="E9" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="F9" s="22"/>
+      <c r="F9" s="25"/>
       <c r="G9" s="17" t="s">
         <v>8</v>
       </c>
@@ -1546,12 +1546,12 @@
       <c r="AO9" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="AP9" s="22"/>
+      <c r="AP9" s="25"/>
       <c r="AQ9" s="17" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="9">
         <v>1</v>
       </c>
@@ -1566,7 +1566,7 @@
         <f>AVERAGE(C10+D10)</f>
         <v>4</v>
       </c>
-      <c r="F10" s="22"/>
+      <c r="F10" s="25"/>
       <c r="G10" s="14"/>
       <c r="H10" s="15"/>
       <c r="I10" s="15">
@@ -1644,13 +1644,13 @@
         <f>AVERAGE(E10+AM10+AN10)/2</f>
         <v>2</v>
       </c>
-      <c r="AP10" s="22"/>
+      <c r="AP10" s="25"/>
       <c r="AQ10" s="15">
         <f>AVERAGE(K10+P10+U10+Z10+AE10+AJ10+AO10)/7</f>
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="9">
         <v>2</v>
       </c>
@@ -1661,7 +1661,7 @@
         <f t="shared" ref="E11:E29" si="0">AVERAGE(C11+D11)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="22"/>
+      <c r="F11" s="25"/>
       <c r="G11" s="14"/>
       <c r="H11" s="15"/>
       <c r="I11" s="15">
@@ -1739,13 +1739,13 @@
         <f t="shared" ref="AO11:AO30" si="14">AVERAGE(E11+AM11+AN11)/2</f>
         <v>0</v>
       </c>
-      <c r="AP11" s="22"/>
+      <c r="AP11" s="25"/>
       <c r="AQ11" s="15">
         <f t="shared" ref="AQ11:AQ30" si="15">AVERAGE(K11+P11+U11+Z11+AE11+AJ11+AO11)/7</f>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="9">
         <v>3</v>
       </c>
@@ -1756,7 +1756,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F12" s="22"/>
+      <c r="F12" s="25"/>
       <c r="G12" s="14"/>
       <c r="H12" s="15"/>
       <c r="I12" s="15">
@@ -1834,13 +1834,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP12" s="22"/>
+      <c r="AP12" s="25"/>
       <c r="AQ12" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A13" s="9">
         <v>4</v>
       </c>
@@ -1851,7 +1851,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F13" s="22"/>
+      <c r="F13" s="25"/>
       <c r="G13" s="14"/>
       <c r="H13" s="15"/>
       <c r="I13" s="15">
@@ -1929,13 +1929,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP13" s="22"/>
+      <c r="AP13" s="25"/>
       <c r="AQ13" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="9">
         <v>5</v>
       </c>
@@ -1946,7 +1946,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F14" s="22"/>
+      <c r="F14" s="25"/>
       <c r="G14" s="14"/>
       <c r="H14" s="15"/>
       <c r="I14" s="15">
@@ -2024,13 +2024,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP14" s="22"/>
+      <c r="AP14" s="25"/>
       <c r="AQ14" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="9">
         <v>6</v>
       </c>
@@ -2041,7 +2041,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F15" s="22"/>
+      <c r="F15" s="25"/>
       <c r="G15" s="14"/>
       <c r="H15" s="15"/>
       <c r="I15" s="15">
@@ -2119,13 +2119,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP15" s="22"/>
+      <c r="AP15" s="25"/>
       <c r="AQ15" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="9">
         <v>7</v>
       </c>
@@ -2136,7 +2136,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F16" s="22"/>
+      <c r="F16" s="25"/>
       <c r="G16" s="14"/>
       <c r="H16" s="15"/>
       <c r="I16" s="15">
@@ -2214,13 +2214,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP16" s="22"/>
+      <c r="AP16" s="25"/>
       <c r="AQ16" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="9">
         <v>8</v>
       </c>
@@ -2231,7 +2231,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F17" s="22"/>
+      <c r="F17" s="25"/>
       <c r="G17" s="14"/>
       <c r="H17" s="15"/>
       <c r="I17" s="15">
@@ -2309,13 +2309,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP17" s="22"/>
+      <c r="AP17" s="25"/>
       <c r="AQ17" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="9">
         <v>9</v>
       </c>
@@ -2326,7 +2326,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F18" s="22"/>
+      <c r="F18" s="25"/>
       <c r="G18" s="14"/>
       <c r="H18" s="15"/>
       <c r="I18" s="15">
@@ -2404,13 +2404,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP18" s="22"/>
+      <c r="AP18" s="25"/>
       <c r="AQ18" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A19" s="9">
         <v>10</v>
       </c>
@@ -2421,7 +2421,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F19" s="22"/>
+      <c r="F19" s="25"/>
       <c r="G19" s="14"/>
       <c r="H19" s="15"/>
       <c r="I19" s="15">
@@ -2499,13 +2499,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP19" s="22"/>
+      <c r="AP19" s="25"/>
       <c r="AQ19" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="9">
         <v>11</v>
       </c>
@@ -2516,7 +2516,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F20" s="22"/>
+      <c r="F20" s="25"/>
       <c r="G20" s="14"/>
       <c r="H20" s="15"/>
       <c r="I20" s="15">
@@ -2594,13 +2594,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP20" s="22"/>
+      <c r="AP20" s="25"/>
       <c r="AQ20" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="9">
         <v>12</v>
       </c>
@@ -2611,7 +2611,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F21" s="22"/>
+      <c r="F21" s="25"/>
       <c r="G21" s="14"/>
       <c r="H21" s="15"/>
       <c r="I21" s="15">
@@ -2689,13 +2689,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP21" s="22"/>
+      <c r="AP21" s="25"/>
       <c r="AQ21" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="9">
         <v>13</v>
       </c>
@@ -2706,7 +2706,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F22" s="22"/>
+      <c r="F22" s="25"/>
       <c r="G22" s="14"/>
       <c r="H22" s="15"/>
       <c r="I22" s="15">
@@ -2784,13 +2784,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP22" s="22"/>
+      <c r="AP22" s="25"/>
       <c r="AQ22" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="9">
         <v>14</v>
       </c>
@@ -2801,7 +2801,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F23" s="22"/>
+      <c r="F23" s="25"/>
       <c r="G23" s="14"/>
       <c r="H23" s="15"/>
       <c r="I23" s="15">
@@ -2879,13 +2879,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP23" s="22"/>
+      <c r="AP23" s="25"/>
       <c r="AQ23" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="9">
         <v>15</v>
       </c>
@@ -2896,7 +2896,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F24" s="22"/>
+      <c r="F24" s="25"/>
       <c r="G24" s="14"/>
       <c r="H24" s="15"/>
       <c r="I24" s="15">
@@ -2974,13 +2974,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP24" s="22"/>
+      <c r="AP24" s="25"/>
       <c r="AQ24" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="9">
         <v>16</v>
       </c>
@@ -2991,7 +2991,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F25" s="22"/>
+      <c r="F25" s="25"/>
       <c r="G25" s="14"/>
       <c r="H25" s="15"/>
       <c r="I25" s="15">
@@ -3069,13 +3069,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP25" s="22"/>
+      <c r="AP25" s="25"/>
       <c r="AQ25" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" s="9">
         <v>17</v>
       </c>
@@ -3086,7 +3086,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F26" s="22"/>
+      <c r="F26" s="25"/>
       <c r="G26" s="14"/>
       <c r="H26" s="15"/>
       <c r="I26" s="15">
@@ -3164,13 +3164,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP26" s="22"/>
+      <c r="AP26" s="25"/>
       <c r="AQ26" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="9">
         <v>18</v>
       </c>
@@ -3181,7 +3181,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F27" s="22"/>
+      <c r="F27" s="25"/>
       <c r="G27" s="14"/>
       <c r="H27" s="15"/>
       <c r="I27" s="15">
@@ -3259,13 +3259,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP27" s="22"/>
+      <c r="AP27" s="25"/>
       <c r="AQ27" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="9">
         <v>19</v>
       </c>
@@ -3276,7 +3276,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F28" s="22"/>
+      <c r="F28" s="25"/>
       <c r="G28" s="14"/>
       <c r="H28" s="15"/>
       <c r="I28" s="15">
@@ -3354,13 +3354,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP28" s="22"/>
+      <c r="AP28" s="25"/>
       <c r="AQ28" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:43" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" s="9">
         <v>20</v>
       </c>
@@ -3371,7 +3371,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F29" s="22"/>
+      <c r="F29" s="25"/>
       <c r="G29" s="14"/>
       <c r="H29" s="15"/>
       <c r="I29" s="15">
@@ -3449,13 +3449,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP29" s="22"/>
+      <c r="AP29" s="25"/>
       <c r="AQ29" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A30" s="9">
         <v>21</v>
       </c>
@@ -3466,7 +3466,7 @@
         <f>AVERAGE(C30+D30)</f>
         <v>0</v>
       </c>
-      <c r="F30" s="22"/>
+      <c r="F30" s="25"/>
       <c r="G30" s="14"/>
       <c r="H30" s="15"/>
       <c r="I30" s="15">
@@ -3544,7 +3544,7 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AP30" s="22"/>
+      <c r="AP30" s="25"/>
       <c r="AQ30" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
@@ -3552,6 +3552,11 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="F9:F30"/>
+    <mergeCell ref="AP7:AQ7"/>
+    <mergeCell ref="AP9:AP30"/>
+    <mergeCell ref="AK7:AO7"/>
     <mergeCell ref="A1:B7"/>
     <mergeCell ref="C1:AQ2"/>
     <mergeCell ref="C3:H3"/>
@@ -3568,11 +3573,6 @@
     <mergeCell ref="AA7:AE7"/>
     <mergeCell ref="AF7:AJ7"/>
     <mergeCell ref="W3:AQ5"/>
-    <mergeCell ref="C7:F7"/>
-    <mergeCell ref="F9:F30"/>
-    <mergeCell ref="AP7:AQ7"/>
-    <mergeCell ref="AP9:AP30"/>
-    <mergeCell ref="AK7:AO7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -3583,451 +3583,451 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AX30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.140625" customWidth="1"/>
-    <col min="2" max="2" width="44.42578125" customWidth="1"/>
-    <col min="3" max="3" width="5.85546875" customWidth="1"/>
-    <col min="4" max="4" width="7.28515625" customWidth="1"/>
+    <col min="1" max="1" width="4.109375" customWidth="1"/>
+    <col min="2" max="2" width="44.44140625" customWidth="1"/>
+    <col min="3" max="3" width="5.88671875" customWidth="1"/>
+    <col min="4" max="4" width="7.33203125" customWidth="1"/>
     <col min="5" max="5" width="6" customWidth="1"/>
-    <col min="6" max="6" width="0.7109375" customWidth="1"/>
-    <col min="7" max="7" width="6.85546875" customWidth="1"/>
-    <col min="8" max="8" width="7.85546875" customWidth="1"/>
-    <col min="9" max="9" width="7.140625" customWidth="1"/>
-    <col min="10" max="10" width="7.42578125" customWidth="1"/>
-    <col min="11" max="11" width="6.7109375" style="2" customWidth="1"/>
-    <col min="12" max="12" width="6.85546875" customWidth="1"/>
-    <col min="13" max="13" width="7.85546875" customWidth="1"/>
-    <col min="14" max="14" width="7.140625" customWidth="1"/>
-    <col min="15" max="15" width="7.42578125" customWidth="1"/>
-    <col min="16" max="16" width="6.7109375" customWidth="1"/>
-    <col min="17" max="17" width="6.85546875" style="2" customWidth="1"/>
-    <col min="18" max="18" width="7.85546875" customWidth="1"/>
-    <col min="19" max="19" width="7.140625" customWidth="1"/>
-    <col min="20" max="20" width="7.42578125" customWidth="1"/>
-    <col min="21" max="21" width="6.7109375" customWidth="1"/>
-    <col min="22" max="22" width="6.85546875" customWidth="1"/>
-    <col min="23" max="23" width="7.85546875" style="2" customWidth="1"/>
-    <col min="24" max="24" width="7.140625" customWidth="1"/>
-    <col min="25" max="25" width="7.42578125" customWidth="1"/>
-    <col min="26" max="26" width="6.7109375" customWidth="1"/>
-    <col min="27" max="27" width="6.85546875" customWidth="1"/>
-    <col min="28" max="28" width="7.85546875" customWidth="1"/>
-    <col min="29" max="29" width="7.140625" style="2" customWidth="1"/>
-    <col min="30" max="30" width="7.42578125" customWidth="1"/>
-    <col min="31" max="31" width="6.7109375" customWidth="1"/>
-    <col min="32" max="32" width="6.85546875" customWidth="1"/>
-    <col min="33" max="33" width="7.85546875" customWidth="1"/>
-    <col min="34" max="34" width="7.140625" customWidth="1"/>
-    <col min="35" max="35" width="7.42578125" style="2" customWidth="1"/>
-    <col min="36" max="36" width="6.7109375" customWidth="1"/>
-    <col min="37" max="37" width="6.85546875" customWidth="1"/>
-    <col min="38" max="38" width="7.85546875" customWidth="1"/>
-    <col min="39" max="39" width="7.140625" customWidth="1"/>
-    <col min="40" max="40" width="7.42578125" customWidth="1"/>
-    <col min="41" max="41" width="6.7109375" style="2" customWidth="1"/>
-    <col min="42" max="42" width="6.85546875" customWidth="1"/>
-    <col min="43" max="43" width="7.85546875" customWidth="1"/>
-    <col min="44" max="44" width="7.140625" customWidth="1"/>
-    <col min="45" max="45" width="7.42578125" customWidth="1"/>
-    <col min="46" max="46" width="6.7109375" customWidth="1"/>
-    <col min="47" max="47" width="6.85546875" style="2" customWidth="1"/>
-    <col min="48" max="48" width="7.85546875" customWidth="1"/>
-    <col min="49" max="49" width="0.7109375" customWidth="1"/>
-    <col min="50" max="50" width="10.28515625" customWidth="1"/>
+    <col min="6" max="6" width="0.6640625" customWidth="1"/>
+    <col min="7" max="7" width="6.88671875" customWidth="1"/>
+    <col min="8" max="8" width="7.88671875" customWidth="1"/>
+    <col min="9" max="9" width="7.109375" customWidth="1"/>
+    <col min="10" max="10" width="7.44140625" customWidth="1"/>
+    <col min="11" max="11" width="6.6640625" style="2" customWidth="1"/>
+    <col min="12" max="12" width="6.88671875" customWidth="1"/>
+    <col min="13" max="13" width="7.88671875" customWidth="1"/>
+    <col min="14" max="14" width="7.109375" customWidth="1"/>
+    <col min="15" max="15" width="7.44140625" customWidth="1"/>
+    <col min="16" max="16" width="6.6640625" customWidth="1"/>
+    <col min="17" max="17" width="6.88671875" style="2" customWidth="1"/>
+    <col min="18" max="18" width="7.88671875" customWidth="1"/>
+    <col min="19" max="19" width="7.109375" customWidth="1"/>
+    <col min="20" max="20" width="7.44140625" customWidth="1"/>
+    <col min="21" max="21" width="6.6640625" customWidth="1"/>
+    <col min="22" max="22" width="6.88671875" customWidth="1"/>
+    <col min="23" max="23" width="7.88671875" style="2" customWidth="1"/>
+    <col min="24" max="24" width="7.109375" customWidth="1"/>
+    <col min="25" max="25" width="7.44140625" customWidth="1"/>
+    <col min="26" max="26" width="6.6640625" customWidth="1"/>
+    <col min="27" max="27" width="6.88671875" customWidth="1"/>
+    <col min="28" max="28" width="7.88671875" customWidth="1"/>
+    <col min="29" max="29" width="7.109375" style="2" customWidth="1"/>
+    <col min="30" max="30" width="7.44140625" customWidth="1"/>
+    <col min="31" max="31" width="6.6640625" customWidth="1"/>
+    <col min="32" max="32" width="6.88671875" customWidth="1"/>
+    <col min="33" max="33" width="7.88671875" customWidth="1"/>
+    <col min="34" max="34" width="7.109375" customWidth="1"/>
+    <col min="35" max="35" width="7.44140625" style="2" customWidth="1"/>
+    <col min="36" max="36" width="6.6640625" customWidth="1"/>
+    <col min="37" max="37" width="6.88671875" customWidth="1"/>
+    <col min="38" max="38" width="7.88671875" customWidth="1"/>
+    <col min="39" max="39" width="7.109375" customWidth="1"/>
+    <col min="40" max="40" width="7.44140625" customWidth="1"/>
+    <col min="41" max="41" width="6.6640625" style="2" customWidth="1"/>
+    <col min="42" max="42" width="6.88671875" customWidth="1"/>
+    <col min="43" max="43" width="7.88671875" customWidth="1"/>
+    <col min="44" max="44" width="7.109375" customWidth="1"/>
+    <col min="45" max="45" width="7.44140625" customWidth="1"/>
+    <col min="46" max="46" width="6.6640625" customWidth="1"/>
+    <col min="47" max="47" width="6.88671875" style="2" customWidth="1"/>
+    <col min="48" max="48" width="7.88671875" customWidth="1"/>
+    <col min="49" max="49" width="0.6640625" customWidth="1"/>
+    <col min="50" max="50" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:50" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24"/>
-      <c r="B1" s="24"/>
-      <c r="C1" s="31" t="s">
+    <row r="1" spans="1:50" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="21"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-      <c r="L1" s="31"/>
-      <c r="M1" s="31"/>
-      <c r="N1" s="31"/>
-      <c r="O1" s="31"/>
-      <c r="P1" s="31"/>
-      <c r="Q1" s="31"/>
-      <c r="R1" s="31"/>
-      <c r="S1" s="31"/>
-      <c r="T1" s="31"/>
-      <c r="U1" s="31"/>
-      <c r="V1" s="31"/>
-      <c r="W1" s="31"/>
-      <c r="X1" s="31"/>
-      <c r="Y1" s="31"/>
-      <c r="Z1" s="31"/>
-      <c r="AA1" s="31"/>
-      <c r="AB1" s="31"/>
-      <c r="AC1" s="31"/>
-      <c r="AD1" s="31"/>
-      <c r="AE1" s="31"/>
-      <c r="AF1" s="31"/>
-      <c r="AG1" s="31"/>
-      <c r="AH1" s="31"/>
-      <c r="AI1" s="31"/>
-      <c r="AJ1" s="31"/>
-      <c r="AK1" s="31"/>
-      <c r="AL1" s="31"/>
-      <c r="AM1" s="31"/>
-      <c r="AN1" s="31"/>
-      <c r="AO1" s="31"/>
-      <c r="AP1" s="31"/>
-      <c r="AQ1" s="31"/>
-      <c r="AR1" s="31"/>
-      <c r="AS1" s="31"/>
-      <c r="AT1" s="31"/>
-      <c r="AU1" s="31"/>
-      <c r="AV1" s="31"/>
-      <c r="AW1" s="31"/>
-      <c r="AX1" s="31"/>
-    </row>
-    <row r="2" spans="1:50" x14ac:dyDescent="0.25">
-      <c r="A2" s="24"/>
-      <c r="B2" s="24"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="31"/>
-      <c r="O2" s="31"/>
-      <c r="P2" s="31"/>
-      <c r="Q2" s="31"/>
-      <c r="R2" s="31"/>
-      <c r="S2" s="31"/>
-      <c r="T2" s="31"/>
-      <c r="U2" s="31"/>
-      <c r="V2" s="31"/>
-      <c r="W2" s="31"/>
-      <c r="X2" s="31"/>
-      <c r="Y2" s="31"/>
-      <c r="Z2" s="31"/>
-      <c r="AA2" s="31"/>
-      <c r="AB2" s="31"/>
-      <c r="AC2" s="31"/>
-      <c r="AD2" s="31"/>
-      <c r="AE2" s="31"/>
-      <c r="AF2" s="31"/>
-      <c r="AG2" s="31"/>
-      <c r="AH2" s="31"/>
-      <c r="AI2" s="31"/>
-      <c r="AJ2" s="31"/>
-      <c r="AK2" s="31"/>
-      <c r="AL2" s="31"/>
-      <c r="AM2" s="31"/>
-      <c r="AN2" s="31"/>
-      <c r="AO2" s="31"/>
-      <c r="AP2" s="31"/>
-      <c r="AQ2" s="31"/>
-      <c r="AR2" s="31"/>
-      <c r="AS2" s="31"/>
-      <c r="AT2" s="31"/>
-      <c r="AU2" s="31"/>
-      <c r="AV2" s="31"/>
-      <c r="AW2" s="31"/>
-      <c r="AX2" s="31"/>
-    </row>
-    <row r="3" spans="1:50" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="24"/>
-      <c r="B3" s="24"/>
-      <c r="C3" s="27" t="s">
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
+      <c r="O1" s="30"/>
+      <c r="P1" s="30"/>
+      <c r="Q1" s="30"/>
+      <c r="R1" s="30"/>
+      <c r="S1" s="30"/>
+      <c r="T1" s="30"/>
+      <c r="U1" s="30"/>
+      <c r="V1" s="30"/>
+      <c r="W1" s="30"/>
+      <c r="X1" s="30"/>
+      <c r="Y1" s="30"/>
+      <c r="Z1" s="30"/>
+      <c r="AA1" s="30"/>
+      <c r="AB1" s="30"/>
+      <c r="AC1" s="30"/>
+      <c r="AD1" s="30"/>
+      <c r="AE1" s="30"/>
+      <c r="AF1" s="30"/>
+      <c r="AG1" s="30"/>
+      <c r="AH1" s="30"/>
+      <c r="AI1" s="30"/>
+      <c r="AJ1" s="30"/>
+      <c r="AK1" s="30"/>
+      <c r="AL1" s="30"/>
+      <c r="AM1" s="30"/>
+      <c r="AN1" s="30"/>
+      <c r="AO1" s="30"/>
+      <c r="AP1" s="30"/>
+      <c r="AQ1" s="30"/>
+      <c r="AR1" s="30"/>
+      <c r="AS1" s="30"/>
+      <c r="AT1" s="30"/>
+      <c r="AU1" s="30"/>
+      <c r="AV1" s="30"/>
+      <c r="AW1" s="30"/>
+      <c r="AX1" s="30"/>
+    </row>
+    <row r="2" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="A2" s="21"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
+      <c r="N2" s="30"/>
+      <c r="O2" s="30"/>
+      <c r="P2" s="30"/>
+      <c r="Q2" s="30"/>
+      <c r="R2" s="30"/>
+      <c r="S2" s="30"/>
+      <c r="T2" s="30"/>
+      <c r="U2" s="30"/>
+      <c r="V2" s="30"/>
+      <c r="W2" s="30"/>
+      <c r="X2" s="30"/>
+      <c r="Y2" s="30"/>
+      <c r="Z2" s="30"/>
+      <c r="AA2" s="30"/>
+      <c r="AB2" s="30"/>
+      <c r="AC2" s="30"/>
+      <c r="AD2" s="30"/>
+      <c r="AE2" s="30"/>
+      <c r="AF2" s="30"/>
+      <c r="AG2" s="30"/>
+      <c r="AH2" s="30"/>
+      <c r="AI2" s="30"/>
+      <c r="AJ2" s="30"/>
+      <c r="AK2" s="30"/>
+      <c r="AL2" s="30"/>
+      <c r="AM2" s="30"/>
+      <c r="AN2" s="30"/>
+      <c r="AO2" s="30"/>
+      <c r="AP2" s="30"/>
+      <c r="AQ2" s="30"/>
+      <c r="AR2" s="30"/>
+      <c r="AS2" s="30"/>
+      <c r="AT2" s="30"/>
+      <c r="AU2" s="30"/>
+      <c r="AV2" s="30"/>
+      <c r="AW2" s="30"/>
+      <c r="AX2" s="30"/>
+    </row>
+    <row r="3" spans="1:50" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="21"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="27"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="27"/>
-      <c r="J3" s="27"/>
-      <c r="K3" s="27"/>
-      <c r="L3" s="27"/>
-      <c r="M3" s="27"/>
-      <c r="N3" s="27"/>
-      <c r="O3" s="27"/>
-      <c r="P3" s="27"/>
-      <c r="Q3" s="27"/>
-      <c r="R3" s="27"/>
-      <c r="S3" s="27"/>
-      <c r="T3" s="27"/>
-      <c r="U3" s="27"/>
-      <c r="V3" s="27"/>
-      <c r="W3" s="28" t="s">
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="24"/>
+      <c r="L3" s="24"/>
+      <c r="M3" s="24"/>
+      <c r="N3" s="24"/>
+      <c r="O3" s="24"/>
+      <c r="P3" s="24"/>
+      <c r="Q3" s="24"/>
+      <c r="R3" s="24"/>
+      <c r="S3" s="24"/>
+      <c r="T3" s="24"/>
+      <c r="U3" s="24"/>
+      <c r="V3" s="24"/>
+      <c r="W3" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="X3" s="29"/>
-      <c r="Y3" s="29"/>
-      <c r="Z3" s="29"/>
-      <c r="AA3" s="29"/>
-      <c r="AB3" s="29"/>
-      <c r="AC3" s="29"/>
-      <c r="AD3" s="29"/>
-      <c r="AE3" s="29"/>
-      <c r="AF3" s="29"/>
-      <c r="AG3" s="29"/>
-      <c r="AH3" s="29"/>
-      <c r="AI3" s="29"/>
-      <c r="AJ3" s="29"/>
-      <c r="AK3" s="29"/>
-      <c r="AL3" s="29"/>
-      <c r="AM3" s="29"/>
-      <c r="AN3" s="29"/>
-      <c r="AO3" s="29"/>
-      <c r="AP3" s="29"/>
-      <c r="AQ3" s="29"/>
-      <c r="AR3" s="29"/>
-      <c r="AS3" s="29"/>
-      <c r="AT3" s="29"/>
-      <c r="AU3" s="29"/>
-      <c r="AV3" s="29"/>
-      <c r="AW3" s="29"/>
-      <c r="AX3" s="29"/>
-    </row>
-    <row r="4" spans="1:50" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="24"/>
-      <c r="B4" s="24"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
-      <c r="K4" s="27"/>
-      <c r="L4" s="27"/>
-      <c r="M4" s="27"/>
-      <c r="N4" s="27"/>
-      <c r="O4" s="27"/>
-      <c r="P4" s="27"/>
-      <c r="Q4" s="27"/>
-      <c r="R4" s="27"/>
-      <c r="S4" s="27"/>
-      <c r="T4" s="27"/>
-      <c r="U4" s="27"/>
-      <c r="V4" s="27"/>
-      <c r="W4" s="29"/>
-      <c r="X4" s="29"/>
-      <c r="Y4" s="29"/>
-      <c r="Z4" s="29"/>
-      <c r="AA4" s="29"/>
-      <c r="AB4" s="29"/>
-      <c r="AC4" s="29"/>
-      <c r="AD4" s="29"/>
-      <c r="AE4" s="29"/>
-      <c r="AF4" s="29"/>
-      <c r="AG4" s="29"/>
-      <c r="AH4" s="29"/>
-      <c r="AI4" s="29"/>
-      <c r="AJ4" s="29"/>
-      <c r="AK4" s="29"/>
-      <c r="AL4" s="29"/>
-      <c r="AM4" s="29"/>
-      <c r="AN4" s="29"/>
-      <c r="AO4" s="29"/>
-      <c r="AP4" s="29"/>
-      <c r="AQ4" s="29"/>
-      <c r="AR4" s="29"/>
-      <c r="AS4" s="29"/>
-      <c r="AT4" s="29"/>
-      <c r="AU4" s="29"/>
-      <c r="AV4" s="29"/>
-      <c r="AW4" s="29"/>
-      <c r="AX4" s="29"/>
-    </row>
-    <row r="5" spans="1:50" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="24"/>
-      <c r="B5" s="24"/>
-      <c r="C5" s="27" t="s">
+      <c r="X3" s="28"/>
+      <c r="Y3" s="28"/>
+      <c r="Z3" s="28"/>
+      <c r="AA3" s="28"/>
+      <c r="AB3" s="28"/>
+      <c r="AC3" s="28"/>
+      <c r="AD3" s="28"/>
+      <c r="AE3" s="28"/>
+      <c r="AF3" s="28"/>
+      <c r="AG3" s="28"/>
+      <c r="AH3" s="28"/>
+      <c r="AI3" s="28"/>
+      <c r="AJ3" s="28"/>
+      <c r="AK3" s="28"/>
+      <c r="AL3" s="28"/>
+      <c r="AM3" s="28"/>
+      <c r="AN3" s="28"/>
+      <c r="AO3" s="28"/>
+      <c r="AP3" s="28"/>
+      <c r="AQ3" s="28"/>
+      <c r="AR3" s="28"/>
+      <c r="AS3" s="28"/>
+      <c r="AT3" s="28"/>
+      <c r="AU3" s="28"/>
+      <c r="AV3" s="28"/>
+      <c r="AW3" s="28"/>
+      <c r="AX3" s="28"/>
+    </row>
+    <row r="4" spans="1:50" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="21"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
+      <c r="P4" s="24"/>
+      <c r="Q4" s="24"/>
+      <c r="R4" s="24"/>
+      <c r="S4" s="24"/>
+      <c r="T4" s="24"/>
+      <c r="U4" s="24"/>
+      <c r="V4" s="24"/>
+      <c r="W4" s="28"/>
+      <c r="X4" s="28"/>
+      <c r="Y4" s="28"/>
+      <c r="Z4" s="28"/>
+      <c r="AA4" s="28"/>
+      <c r="AB4" s="28"/>
+      <c r="AC4" s="28"/>
+      <c r="AD4" s="28"/>
+      <c r="AE4" s="28"/>
+      <c r="AF4" s="28"/>
+      <c r="AG4" s="28"/>
+      <c r="AH4" s="28"/>
+      <c r="AI4" s="28"/>
+      <c r="AJ4" s="28"/>
+      <c r="AK4" s="28"/>
+      <c r="AL4" s="28"/>
+      <c r="AM4" s="28"/>
+      <c r="AN4" s="28"/>
+      <c r="AO4" s="28"/>
+      <c r="AP4" s="28"/>
+      <c r="AQ4" s="28"/>
+      <c r="AR4" s="28"/>
+      <c r="AS4" s="28"/>
+      <c r="AT4" s="28"/>
+      <c r="AU4" s="28"/>
+      <c r="AV4" s="28"/>
+      <c r="AW4" s="28"/>
+      <c r="AX4" s="28"/>
+    </row>
+    <row r="5" spans="1:50" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="21"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
-      <c r="K5" s="27"/>
-      <c r="L5" s="27"/>
-      <c r="M5" s="27"/>
-      <c r="N5" s="27"/>
-      <c r="O5" s="27"/>
-      <c r="P5" s="27"/>
-      <c r="Q5" s="27"/>
-      <c r="R5" s="27"/>
-      <c r="S5" s="27"/>
-      <c r="T5" s="27"/>
-      <c r="U5" s="27"/>
-      <c r="V5" s="27"/>
-      <c r="W5" s="29"/>
-      <c r="X5" s="29"/>
-      <c r="Y5" s="29"/>
-      <c r="Z5" s="29"/>
-      <c r="AA5" s="29"/>
-      <c r="AB5" s="29"/>
-      <c r="AC5" s="29"/>
-      <c r="AD5" s="29"/>
-      <c r="AE5" s="29"/>
-      <c r="AF5" s="29"/>
-      <c r="AG5" s="29"/>
-      <c r="AH5" s="29"/>
-      <c r="AI5" s="29"/>
-      <c r="AJ5" s="29"/>
-      <c r="AK5" s="29"/>
-      <c r="AL5" s="29"/>
-      <c r="AM5" s="29"/>
-      <c r="AN5" s="29"/>
-      <c r="AO5" s="29"/>
-      <c r="AP5" s="29"/>
-      <c r="AQ5" s="29"/>
-      <c r="AR5" s="29"/>
-      <c r="AS5" s="29"/>
-      <c r="AT5" s="29"/>
-      <c r="AU5" s="29"/>
-      <c r="AV5" s="29"/>
-      <c r="AW5" s="29"/>
-      <c r="AX5" s="29"/>
-    </row>
-    <row r="6" spans="1:50" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="24"/>
-      <c r="B6" s="24"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
-      <c r="M6" s="22"/>
-      <c r="N6" s="22"/>
-      <c r="O6" s="22"/>
-      <c r="P6" s="22"/>
-      <c r="Q6" s="22"/>
-      <c r="R6" s="22"/>
-      <c r="S6" s="22"/>
-      <c r="T6" s="22"/>
-      <c r="U6" s="22"/>
-      <c r="V6" s="22"/>
-      <c r="W6" s="22"/>
-      <c r="X6" s="22"/>
-      <c r="Y6" s="22"/>
-      <c r="Z6" s="22"/>
-      <c r="AA6" s="22"/>
-      <c r="AB6" s="22"/>
-      <c r="AC6" s="22"/>
-      <c r="AD6" s="22"/>
-      <c r="AE6" s="22"/>
-      <c r="AF6" s="22"/>
-      <c r="AG6" s="22"/>
-      <c r="AH6" s="22"/>
-      <c r="AI6" s="22"/>
-      <c r="AJ6" s="22"/>
-      <c r="AK6" s="22"/>
-      <c r="AL6" s="22"/>
-      <c r="AM6" s="22"/>
-      <c r="AN6" s="22"/>
-      <c r="AO6" s="22"/>
-      <c r="AP6" s="22"/>
-      <c r="AQ6" s="22"/>
-      <c r="AR6" s="22"/>
-      <c r="AS6" s="22"/>
-      <c r="AT6" s="22"/>
-      <c r="AU6" s="22"/>
-      <c r="AV6" s="22"/>
-      <c r="AW6" s="22"/>
-      <c r="AX6" s="22"/>
-    </row>
-    <row r="7" spans="1:50" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="24"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="21" t="s">
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="24"/>
+      <c r="M5" s="24"/>
+      <c r="N5" s="24"/>
+      <c r="O5" s="24"/>
+      <c r="P5" s="24"/>
+      <c r="Q5" s="24"/>
+      <c r="R5" s="24"/>
+      <c r="S5" s="24"/>
+      <c r="T5" s="24"/>
+      <c r="U5" s="24"/>
+      <c r="V5" s="24"/>
+      <c r="W5" s="28"/>
+      <c r="X5" s="28"/>
+      <c r="Y5" s="28"/>
+      <c r="Z5" s="28"/>
+      <c r="AA5" s="28"/>
+      <c r="AB5" s="28"/>
+      <c r="AC5" s="28"/>
+      <c r="AD5" s="28"/>
+      <c r="AE5" s="28"/>
+      <c r="AF5" s="28"/>
+      <c r="AG5" s="28"/>
+      <c r="AH5" s="28"/>
+      <c r="AI5" s="28"/>
+      <c r="AJ5" s="28"/>
+      <c r="AK5" s="28"/>
+      <c r="AL5" s="28"/>
+      <c r="AM5" s="28"/>
+      <c r="AN5" s="28"/>
+      <c r="AO5" s="28"/>
+      <c r="AP5" s="28"/>
+      <c r="AQ5" s="28"/>
+      <c r="AR5" s="28"/>
+      <c r="AS5" s="28"/>
+      <c r="AT5" s="28"/>
+      <c r="AU5" s="28"/>
+      <c r="AV5" s="28"/>
+      <c r="AW5" s="28"/>
+      <c r="AX5" s="28"/>
+    </row>
+    <row r="6" spans="1:50" ht="6.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="21"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="25"/>
+      <c r="J6" s="25"/>
+      <c r="K6" s="25"/>
+      <c r="L6" s="25"/>
+      <c r="M6" s="25"/>
+      <c r="N6" s="25"/>
+      <c r="O6" s="25"/>
+      <c r="P6" s="25"/>
+      <c r="Q6" s="25"/>
+      <c r="R6" s="25"/>
+      <c r="S6" s="25"/>
+      <c r="T6" s="25"/>
+      <c r="U6" s="25"/>
+      <c r="V6" s="25"/>
+      <c r="W6" s="25"/>
+      <c r="X6" s="25"/>
+      <c r="Y6" s="25"/>
+      <c r="Z6" s="25"/>
+      <c r="AA6" s="25"/>
+      <c r="AB6" s="25"/>
+      <c r="AC6" s="25"/>
+      <c r="AD6" s="25"/>
+      <c r="AE6" s="25"/>
+      <c r="AF6" s="25"/>
+      <c r="AG6" s="25"/>
+      <c r="AH6" s="25"/>
+      <c r="AI6" s="25"/>
+      <c r="AJ6" s="25"/>
+      <c r="AK6" s="25"/>
+      <c r="AL6" s="25"/>
+      <c r="AM6" s="25"/>
+      <c r="AN6" s="25"/>
+      <c r="AO6" s="25"/>
+      <c r="AP6" s="25"/>
+      <c r="AQ6" s="25"/>
+      <c r="AR6" s="25"/>
+      <c r="AS6" s="25"/>
+      <c r="AT6" s="25"/>
+      <c r="AU6" s="25"/>
+      <c r="AV6" s="25"/>
+      <c r="AW6" s="25"/>
+      <c r="AX6" s="25"/>
+    </row>
+    <row r="7" spans="1:50" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="21"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="21" t="s">
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="H7" s="21"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="21"/>
-      <c r="M7" s="21" t="s">
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="26"/>
+      <c r="M7" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="N7" s="21"/>
-      <c r="O7" s="21"/>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="21"/>
-      <c r="S7" s="21" t="s">
+      <c r="N7" s="26"/>
+      <c r="O7" s="26"/>
+      <c r="P7" s="26"/>
+      <c r="Q7" s="26"/>
+      <c r="R7" s="26"/>
+      <c r="S7" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="T7" s="21"/>
-      <c r="U7" s="21"/>
-      <c r="V7" s="21"/>
-      <c r="W7" s="21"/>
-      <c r="X7" s="21"/>
-      <c r="Y7" s="21" t="s">
+      <c r="T7" s="26"/>
+      <c r="U7" s="26"/>
+      <c r="V7" s="26"/>
+      <c r="W7" s="26"/>
+      <c r="X7" s="26"/>
+      <c r="Y7" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="Z7" s="21"/>
-      <c r="AA7" s="21"/>
-      <c r="AB7" s="21"/>
-      <c r="AC7" s="21"/>
-      <c r="AD7" s="21"/>
-      <c r="AE7" s="21" t="s">
+      <c r="Z7" s="26"/>
+      <c r="AA7" s="26"/>
+      <c r="AB7" s="26"/>
+      <c r="AC7" s="26"/>
+      <c r="AD7" s="26"/>
+      <c r="AE7" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="AF7" s="21"/>
-      <c r="AG7" s="21"/>
-      <c r="AH7" s="21"/>
-      <c r="AI7" s="21"/>
-      <c r="AJ7" s="21"/>
-      <c r="AK7" s="21" t="s">
+      <c r="AF7" s="26"/>
+      <c r="AG7" s="26"/>
+      <c r="AH7" s="26"/>
+      <c r="AI7" s="26"/>
+      <c r="AJ7" s="26"/>
+      <c r="AK7" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="AL7" s="21"/>
-      <c r="AM7" s="21"/>
-      <c r="AN7" s="21"/>
-      <c r="AO7" s="21"/>
-      <c r="AP7" s="21"/>
-      <c r="AQ7" s="21" t="s">
+      <c r="AL7" s="26"/>
+      <c r="AM7" s="26"/>
+      <c r="AN7" s="26"/>
+      <c r="AO7" s="26"/>
+      <c r="AP7" s="26"/>
+      <c r="AQ7" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="AR7" s="21"/>
-      <c r="AS7" s="21"/>
-      <c r="AT7" s="21"/>
-      <c r="AU7" s="21"/>
-      <c r="AV7" s="21"/>
-      <c r="AW7" s="23" t="s">
+      <c r="AR7" s="26"/>
+      <c r="AS7" s="26"/>
+      <c r="AT7" s="26"/>
+      <c r="AU7" s="26"/>
+      <c r="AV7" s="26"/>
+      <c r="AW7" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="AX7" s="23"/>
-    </row>
-    <row r="8" spans="1:50" ht="0.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AX7" s="29"/>
+    </row>
+    <row r="8" spans="1:50" ht="0.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -4079,7 +4079,7 @@
       <c r="AW8" s="5"/>
       <c r="AX8" s="5"/>
     </row>
-    <row r="9" spans="1:50" ht="97.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:50" ht="97.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>0</v>
       </c>
@@ -4095,7 +4095,7 @@
       <c r="E9" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="F9" s="30"/>
+      <c r="F9" s="31"/>
       <c r="G9" s="17" t="s">
         <v>8</v>
       </c>
@@ -4222,12 +4222,12 @@
       <c r="AV9" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="AW9" s="22"/>
+      <c r="AW9" s="25"/>
       <c r="AX9" s="17" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="9">
         <v>1</v>
       </c>
@@ -4242,7 +4242,7 @@
         <f>AVERAGE(C10+D10)</f>
         <v>4</v>
       </c>
-      <c r="F10" s="30"/>
+      <c r="F10" s="31"/>
       <c r="G10" s="14"/>
       <c r="H10" s="15"/>
       <c r="I10" s="15">
@@ -4327,13 +4327,13 @@
         <f>AVERAGE(E10+AS10+AT10+AU10)/3</f>
         <v>1.3333333333333333</v>
       </c>
-      <c r="AW10" s="22"/>
+      <c r="AW10" s="25"/>
       <c r="AX10" s="15">
         <f>AVERAGE(L10+R10+X10+AD10+AJ10+AP10+AV10)/7</f>
         <v>1.3333333333333333</v>
       </c>
     </row>
-    <row r="11" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="9">
         <v>2</v>
       </c>
@@ -4344,7 +4344,7 @@
         <f t="shared" ref="E11:E29" si="0">AVERAGE(C11+D11)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="30"/>
+      <c r="F11" s="31"/>
       <c r="G11" s="14"/>
       <c r="H11" s="15"/>
       <c r="I11" s="15">
@@ -4429,13 +4429,13 @@
         <f t="shared" ref="AV11:AV30" si="14">AVERAGE(E11+AS11+AT11+AU11)/3</f>
         <v>0</v>
       </c>
-      <c r="AW11" s="22"/>
+      <c r="AW11" s="25"/>
       <c r="AX11" s="15">
         <f t="shared" ref="AX11:AX30" si="15">AVERAGE(L11+R11+X11+AD11+AJ11+AP11+AV11)/7</f>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="9">
         <v>3</v>
       </c>
@@ -4446,7 +4446,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F12" s="30"/>
+      <c r="F12" s="31"/>
       <c r="G12" s="14"/>
       <c r="H12" s="15"/>
       <c r="I12" s="15">
@@ -4531,13 +4531,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW12" s="22"/>
+      <c r="AW12" s="25"/>
       <c r="AX12" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A13" s="9">
         <v>4</v>
       </c>
@@ -4548,7 +4548,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F13" s="30"/>
+      <c r="F13" s="31"/>
       <c r="G13" s="14"/>
       <c r="H13" s="15"/>
       <c r="I13" s="15">
@@ -4633,13 +4633,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW13" s="22"/>
+      <c r="AW13" s="25"/>
       <c r="AX13" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="9">
         <v>5</v>
       </c>
@@ -4650,7 +4650,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F14" s="30"/>
+      <c r="F14" s="31"/>
       <c r="G14" s="14"/>
       <c r="H14" s="15"/>
       <c r="I14" s="15">
@@ -4735,13 +4735,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW14" s="22"/>
+      <c r="AW14" s="25"/>
       <c r="AX14" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="9">
         <v>6</v>
       </c>
@@ -4752,7 +4752,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F15" s="30"/>
+      <c r="F15" s="31"/>
       <c r="G15" s="14"/>
       <c r="H15" s="15"/>
       <c r="I15" s="15">
@@ -4837,13 +4837,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW15" s="22"/>
+      <c r="AW15" s="25"/>
       <c r="AX15" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="9">
         <v>7</v>
       </c>
@@ -4854,7 +4854,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F16" s="30"/>
+      <c r="F16" s="31"/>
       <c r="G16" s="14"/>
       <c r="H16" s="15"/>
       <c r="I16" s="15">
@@ -4939,13 +4939,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW16" s="22"/>
+      <c r="AW16" s="25"/>
       <c r="AX16" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="9">
         <v>8</v>
       </c>
@@ -4956,7 +4956,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F17" s="30"/>
+      <c r="F17" s="31"/>
       <c r="G17" s="14"/>
       <c r="H17" s="15"/>
       <c r="I17" s="15">
@@ -5041,13 +5041,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW17" s="22"/>
+      <c r="AW17" s="25"/>
       <c r="AX17" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="9">
         <v>9</v>
       </c>
@@ -5058,7 +5058,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F18" s="30"/>
+      <c r="F18" s="31"/>
       <c r="G18" s="14"/>
       <c r="H18" s="15"/>
       <c r="I18" s="15">
@@ -5143,13 +5143,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW18" s="22"/>
+      <c r="AW18" s="25"/>
       <c r="AX18" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A19" s="9">
         <v>10</v>
       </c>
@@ -5160,7 +5160,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F19" s="30"/>
+      <c r="F19" s="31"/>
       <c r="G19" s="14"/>
       <c r="H19" s="15"/>
       <c r="I19" s="15">
@@ -5245,13 +5245,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW19" s="22"/>
+      <c r="AW19" s="25"/>
       <c r="AX19" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="9">
         <v>11</v>
       </c>
@@ -5262,7 +5262,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F20" s="30"/>
+      <c r="F20" s="31"/>
       <c r="G20" s="14"/>
       <c r="H20" s="15"/>
       <c r="I20" s="15">
@@ -5347,13 +5347,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW20" s="22"/>
+      <c r="AW20" s="25"/>
       <c r="AX20" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="9">
         <v>12</v>
       </c>
@@ -5364,7 +5364,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F21" s="30"/>
+      <c r="F21" s="31"/>
       <c r="G21" s="14"/>
       <c r="H21" s="15"/>
       <c r="I21" s="15">
@@ -5449,13 +5449,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW21" s="22"/>
+      <c r="AW21" s="25"/>
       <c r="AX21" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="9">
         <v>13</v>
       </c>
@@ -5466,7 +5466,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F22" s="30"/>
+      <c r="F22" s="31"/>
       <c r="G22" s="14"/>
       <c r="H22" s="15"/>
       <c r="I22" s="15">
@@ -5551,13 +5551,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW22" s="22"/>
+      <c r="AW22" s="25"/>
       <c r="AX22" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="9">
         <v>14</v>
       </c>
@@ -5568,7 +5568,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F23" s="30"/>
+      <c r="F23" s="31"/>
       <c r="G23" s="14"/>
       <c r="H23" s="15"/>
       <c r="I23" s="15">
@@ -5653,13 +5653,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW23" s="22"/>
+      <c r="AW23" s="25"/>
       <c r="AX23" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="9">
         <v>15</v>
       </c>
@@ -5670,7 +5670,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F24" s="30"/>
+      <c r="F24" s="31"/>
       <c r="G24" s="14"/>
       <c r="H24" s="15"/>
       <c r="I24" s="15">
@@ -5755,13 +5755,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW24" s="22"/>
+      <c r="AW24" s="25"/>
       <c r="AX24" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="9">
         <v>16</v>
       </c>
@@ -5772,7 +5772,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F25" s="30"/>
+      <c r="F25" s="31"/>
       <c r="G25" s="14"/>
       <c r="H25" s="15"/>
       <c r="I25" s="15">
@@ -5857,13 +5857,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW25" s="22"/>
+      <c r="AW25" s="25"/>
       <c r="AX25" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" s="9">
         <v>17</v>
       </c>
@@ -5874,7 +5874,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F26" s="30"/>
+      <c r="F26" s="31"/>
       <c r="G26" s="14"/>
       <c r="H26" s="15"/>
       <c r="I26" s="15">
@@ -5959,13 +5959,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW26" s="22"/>
+      <c r="AW26" s="25"/>
       <c r="AX26" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="9">
         <v>18</v>
       </c>
@@ -5976,7 +5976,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F27" s="30"/>
+      <c r="F27" s="31"/>
       <c r="G27" s="14"/>
       <c r="H27" s="15"/>
       <c r="I27" s="15">
@@ -6061,13 +6061,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW27" s="22"/>
+      <c r="AW27" s="25"/>
       <c r="AX27" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="9">
         <v>19</v>
       </c>
@@ -6078,7 +6078,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F28" s="30"/>
+      <c r="F28" s="31"/>
       <c r="G28" s="14"/>
       <c r="H28" s="15"/>
       <c r="I28" s="15">
@@ -6163,13 +6163,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW28" s="22"/>
+      <c r="AW28" s="25"/>
       <c r="AX28" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:50" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:50" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" s="9">
         <v>20</v>
       </c>
@@ -6180,7 +6180,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F29" s="30"/>
+      <c r="F29" s="31"/>
       <c r="G29" s="14"/>
       <c r="H29" s="15"/>
       <c r="I29" s="15">
@@ -6265,13 +6265,13 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW29" s="22"/>
+      <c r="AW29" s="25"/>
       <c r="AX29" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A30" s="9">
         <v>21</v>
       </c>
@@ -6282,7 +6282,7 @@
         <f>AVERAGE(C30+D30)</f>
         <v>0</v>
       </c>
-      <c r="F30" s="30"/>
+      <c r="F30" s="31"/>
       <c r="G30" s="14"/>
       <c r="H30" s="15"/>
       <c r="I30" s="15">
@@ -6367,7 +6367,7 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="AW30" s="22"/>
+      <c r="AW30" s="25"/>
       <c r="AX30" s="15">
         <f t="shared" si="15"/>
         <v>0</v>
@@ -6375,6 +6375,15 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="AW9:AW30"/>
+    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="I5:V5"/>
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="F9:F30"/>
+    <mergeCell ref="AQ7:AV7"/>
+    <mergeCell ref="Y7:AD7"/>
+    <mergeCell ref="AE7:AJ7"/>
+    <mergeCell ref="AK7:AP7"/>
     <mergeCell ref="A1:B7"/>
     <mergeCell ref="C3:H3"/>
     <mergeCell ref="I3:V3"/>
@@ -6387,15 +6396,6 @@
     <mergeCell ref="W3:AX5"/>
     <mergeCell ref="C6:AX6"/>
     <mergeCell ref="AW7:AX7"/>
-    <mergeCell ref="AW9:AW30"/>
-    <mergeCell ref="C5:H5"/>
-    <mergeCell ref="I5:V5"/>
-    <mergeCell ref="C7:F7"/>
-    <mergeCell ref="F9:F30"/>
-    <mergeCell ref="AQ7:AV7"/>
-    <mergeCell ref="Y7:AD7"/>
-    <mergeCell ref="AE7:AJ7"/>
-    <mergeCell ref="AK7:AP7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6405,137 +6405,137 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:V30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.28515625" customWidth="1"/>
-    <col min="2" max="2" width="53.42578125" customWidth="1"/>
+    <col min="1" max="1" width="5.33203125" customWidth="1"/>
+    <col min="2" max="2" width="53.44140625" customWidth="1"/>
     <col min="3" max="3" width="3" customWidth="1"/>
-    <col min="11" max="11" width="1.5703125" customWidth="1"/>
+    <col min="11" max="11" width="1.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A1" s="24"/>
-      <c r="B1" s="24"/>
+    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A1" s="21"/>
+      <c r="B1" s="21"/>
       <c r="C1" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-    </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A2" s="24"/>
-      <c r="B2" s="24"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-    </row>
-    <row r="3" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="24"/>
-      <c r="B3" s="24"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27" t="s">
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A2" s="21"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23"/>
+    </row>
+    <row r="3" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="21"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="27"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="27"/>
-      <c r="J3" s="27"/>
-      <c r="K3" s="27"/>
-      <c r="L3" s="27"/>
-      <c r="M3" s="27"/>
-      <c r="N3" s="27"/>
-      <c r="O3" s="27"/>
-      <c r="P3" s="27"/>
-      <c r="Q3" s="27"/>
-      <c r="R3" s="27"/>
-      <c r="S3" s="27"/>
-      <c r="T3" s="27"/>
-      <c r="U3" s="27"/>
-      <c r="V3" s="27"/>
-    </row>
-    <row r="4" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="24"/>
-      <c r="B4" s="24"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
-      <c r="K4" s="27"/>
-      <c r="L4" s="27"/>
-      <c r="M4" s="27"/>
-      <c r="N4" s="27"/>
-      <c r="O4" s="27"/>
-      <c r="P4" s="27"/>
-      <c r="Q4" s="27"/>
-      <c r="R4" s="27"/>
-      <c r="S4" s="27"/>
-      <c r="T4" s="27"/>
-      <c r="U4" s="27"/>
-      <c r="V4" s="27"/>
-    </row>
-    <row r="5" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="24"/>
-      <c r="B5" s="24"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27" t="s">
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="24"/>
+      <c r="L3" s="24"/>
+      <c r="M3" s="24"/>
+      <c r="N3" s="24"/>
+      <c r="O3" s="24"/>
+      <c r="P3" s="24"/>
+      <c r="Q3" s="24"/>
+      <c r="R3" s="24"/>
+      <c r="S3" s="24"/>
+      <c r="T3" s="24"/>
+      <c r="U3" s="24"/>
+      <c r="V3" s="24"/>
+    </row>
+    <row r="4" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="21"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
+      <c r="P4" s="24"/>
+      <c r="Q4" s="24"/>
+      <c r="R4" s="24"/>
+      <c r="S4" s="24"/>
+      <c r="T4" s="24"/>
+      <c r="U4" s="24"/>
+      <c r="V4" s="24"/>
+    </row>
+    <row r="5" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="21"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
-      <c r="K5" s="27"/>
-      <c r="L5" s="27"/>
-      <c r="M5" s="27"/>
-      <c r="N5" s="27"/>
-      <c r="O5" s="27"/>
-      <c r="P5" s="27"/>
-      <c r="Q5" s="27"/>
-      <c r="R5" s="27"/>
-      <c r="S5" s="27"/>
-      <c r="T5" s="27"/>
-      <c r="U5" s="27"/>
-      <c r="V5" s="27"/>
-    </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A6" s="24"/>
-      <c r="B6" s="24"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
-    </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A7" s="24"/>
-      <c r="B7" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="24"/>
+      <c r="M5" s="24"/>
+      <c r="N5" s="24"/>
+      <c r="O5" s="24"/>
+      <c r="P5" s="24"/>
+      <c r="Q5" s="24"/>
+      <c r="R5" s="24"/>
+      <c r="S5" s="24"/>
+      <c r="T5" s="24"/>
+      <c r="U5" s="24"/>
+      <c r="V5" s="24"/>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A6" s="21"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="25"/>
+      <c r="J6" s="25"/>
+      <c r="K6" s="25"/>
+      <c r="L6" s="25"/>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A7" s="21"/>
+      <c r="B7" s="21"/>
       <c r="C7" s="16"/>
       <c r="D7" s="16" t="s">
         <v>37</v>
@@ -6558,12 +6558,12 @@
       <c r="J7" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="K7" s="23" t="s">
+      <c r="K7" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="L7" s="23"/>
-    </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="L7" s="29"/>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -6577,14 +6577,14 @@
       <c r="K8" s="5"/>
       <c r="L8" s="5"/>
     </row>
-    <row r="9" spans="1:22" ht="30.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" ht="28.2" x14ac:dyDescent="0.3">
       <c r="A9" s="16" t="s">
         <v>0</v>
       </c>
       <c r="B9" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C9" s="22"/>
+      <c r="C9" s="25"/>
       <c r="D9" s="20" t="s">
         <v>38</v>
       </c>
@@ -6606,17 +6606,17 @@
       <c r="J9" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="K9" s="22"/>
+      <c r="K9" s="25"/>
       <c r="L9" s="19" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="16">
         <v>1</v>
       </c>
       <c r="B10" s="3"/>
-      <c r="C10" s="22"/>
+      <c r="C10" s="25"/>
       <c r="D10" s="14">
         <v>8</v>
       </c>
@@ -6638,18 +6638,18 @@
       <c r="J10" s="14">
         <v>9</v>
       </c>
-      <c r="K10" s="22"/>
+      <c r="K10" s="25"/>
       <c r="L10" s="15">
         <f>AVERAGE(D10+E10+F10+G10+H10+I10+J10)/7</f>
         <v>8.7142857142857135</v>
       </c>
     </row>
-    <row r="11" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="16">
         <v>2</v>
       </c>
       <c r="B11" s="3"/>
-      <c r="C11" s="22"/>
+      <c r="C11" s="25"/>
       <c r="D11" s="14"/>
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
@@ -6657,18 +6657,18 @@
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
       <c r="J11" s="14"/>
-      <c r="K11" s="22"/>
+      <c r="K11" s="25"/>
       <c r="L11" s="15">
         <f t="shared" ref="L11:L30" si="0">AVERAGE(D11+E11+F11+G11+H11+I11+J11)/7</f>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="16">
         <v>3</v>
       </c>
       <c r="B12" s="3"/>
-      <c r="C12" s="22"/>
+      <c r="C12" s="25"/>
       <c r="D12" s="14"/>
       <c r="E12" s="14"/>
       <c r="F12" s="14"/>
@@ -6676,18 +6676,18 @@
       <c r="H12" s="14"/>
       <c r="I12" s="14"/>
       <c r="J12" s="14"/>
-      <c r="K12" s="22"/>
+      <c r="K12" s="25"/>
       <c r="L12" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A13" s="16">
         <v>4</v>
       </c>
       <c r="B13" s="4"/>
-      <c r="C13" s="22"/>
+      <c r="C13" s="25"/>
       <c r="D13" s="14"/>
       <c r="E13" s="14"/>
       <c r="F13" s="14"/>
@@ -6695,18 +6695,18 @@
       <c r="H13" s="14"/>
       <c r="I13" s="14"/>
       <c r="J13" s="14"/>
-      <c r="K13" s="22"/>
+      <c r="K13" s="25"/>
       <c r="L13" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:22" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="16">
         <v>5</v>
       </c>
       <c r="B14" s="3"/>
-      <c r="C14" s="22"/>
+      <c r="C14" s="25"/>
       <c r="D14" s="14"/>
       <c r="E14" s="14"/>
       <c r="F14" s="14"/>
@@ -6714,18 +6714,18 @@
       <c r="H14" s="14"/>
       <c r="I14" s="14"/>
       <c r="J14" s="14"/>
-      <c r="K14" s="22"/>
+      <c r="K14" s="25"/>
       <c r="L14" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:22" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="16">
         <v>6</v>
       </c>
       <c r="B15" s="3"/>
-      <c r="C15" s="22"/>
+      <c r="C15" s="25"/>
       <c r="D15" s="14"/>
       <c r="E15" s="14"/>
       <c r="F15" s="14"/>
@@ -6733,18 +6733,18 @@
       <c r="H15" s="14"/>
       <c r="I15" s="14"/>
       <c r="J15" s="14"/>
-      <c r="K15" s="22"/>
+      <c r="K15" s="25"/>
       <c r="L15" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:22" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="16">
         <v>7</v>
       </c>
       <c r="B16" s="3"/>
-      <c r="C16" s="22"/>
+      <c r="C16" s="25"/>
       <c r="D16" s="14"/>
       <c r="E16" s="14"/>
       <c r="F16" s="14"/>
@@ -6752,18 +6752,18 @@
       <c r="H16" s="14"/>
       <c r="I16" s="14"/>
       <c r="J16" s="14"/>
-      <c r="K16" s="22"/>
+      <c r="K16" s="25"/>
       <c r="L16" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="16">
         <v>8</v>
       </c>
       <c r="B17" s="6"/>
-      <c r="C17" s="22"/>
+      <c r="C17" s="25"/>
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
       <c r="F17" s="14"/>
@@ -6771,18 +6771,18 @@
       <c r="H17" s="14"/>
       <c r="I17" s="14"/>
       <c r="J17" s="14"/>
-      <c r="K17" s="22"/>
+      <c r="K17" s="25"/>
       <c r="L17" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="16">
         <v>9</v>
       </c>
       <c r="B18" s="3"/>
-      <c r="C18" s="22"/>
+      <c r="C18" s="25"/>
       <c r="D18" s="14"/>
       <c r="E18" s="14"/>
       <c r="F18" s="14"/>
@@ -6790,18 +6790,18 @@
       <c r="H18" s="14"/>
       <c r="I18" s="14"/>
       <c r="J18" s="14"/>
-      <c r="K18" s="22"/>
+      <c r="K18" s="25"/>
       <c r="L18" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="16">
         <v>10</v>
       </c>
       <c r="B19" s="5"/>
-      <c r="C19" s="22"/>
+      <c r="C19" s="25"/>
       <c r="D19" s="14"/>
       <c r="E19" s="14"/>
       <c r="F19" s="14"/>
@@ -6809,18 +6809,18 @@
       <c r="H19" s="14"/>
       <c r="I19" s="14"/>
       <c r="J19" s="14"/>
-      <c r="K19" s="22"/>
+      <c r="K19" s="25"/>
       <c r="L19" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="16">
         <v>11</v>
       </c>
       <c r="B20" s="3"/>
-      <c r="C20" s="22"/>
+      <c r="C20" s="25"/>
       <c r="D20" s="14"/>
       <c r="E20" s="14"/>
       <c r="F20" s="14"/>
@@ -6828,18 +6828,18 @@
       <c r="H20" s="14"/>
       <c r="I20" s="14"/>
       <c r="J20" s="14"/>
-      <c r="K20" s="22"/>
+      <c r="K20" s="25"/>
       <c r="L20" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="16">
         <v>12</v>
       </c>
       <c r="B21" s="7"/>
-      <c r="C21" s="22"/>
+      <c r="C21" s="25"/>
       <c r="D21" s="14"/>
       <c r="E21" s="14"/>
       <c r="F21" s="14"/>
@@ -6847,18 +6847,18 @@
       <c r="H21" s="14"/>
       <c r="I21" s="14"/>
       <c r="J21" s="14"/>
-      <c r="K21" s="22"/>
+      <c r="K21" s="25"/>
       <c r="L21" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="16">
         <v>13</v>
       </c>
       <c r="B22" s="3"/>
-      <c r="C22" s="22"/>
+      <c r="C22" s="25"/>
       <c r="D22" s="14"/>
       <c r="E22" s="14"/>
       <c r="F22" s="14"/>
@@ -6866,18 +6866,18 @@
       <c r="H22" s="14"/>
       <c r="I22" s="14"/>
       <c r="J22" s="14"/>
-      <c r="K22" s="22"/>
+      <c r="K22" s="25"/>
       <c r="L22" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="16">
         <v>14</v>
       </c>
       <c r="B23" s="7"/>
-      <c r="C23" s="22"/>
+      <c r="C23" s="25"/>
       <c r="D23" s="14"/>
       <c r="E23" s="14"/>
       <c r="F23" s="14"/>
@@ -6885,18 +6885,18 @@
       <c r="H23" s="14"/>
       <c r="I23" s="14"/>
       <c r="J23" s="14"/>
-      <c r="K23" s="22"/>
+      <c r="K23" s="25"/>
       <c r="L23" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="16">
         <v>15</v>
       </c>
       <c r="B24" s="3"/>
-      <c r="C24" s="22"/>
+      <c r="C24" s="25"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
       <c r="F24" s="14"/>
@@ -6904,18 +6904,18 @@
       <c r="H24" s="14"/>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
-      <c r="K24" s="22"/>
+      <c r="K24" s="25"/>
       <c r="L24" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="16">
         <v>16</v>
       </c>
       <c r="B25" s="3"/>
-      <c r="C25" s="22"/>
+      <c r="C25" s="25"/>
       <c r="D25" s="14"/>
       <c r="E25" s="14"/>
       <c r="F25" s="14"/>
@@ -6923,18 +6923,18 @@
       <c r="H25" s="14"/>
       <c r="I25" s="14"/>
       <c r="J25" s="14"/>
-      <c r="K25" s="22"/>
+      <c r="K25" s="25"/>
       <c r="L25" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" s="16">
         <v>17</v>
       </c>
       <c r="B26" s="3"/>
-      <c r="C26" s="22"/>
+      <c r="C26" s="25"/>
       <c r="D26" s="14"/>
       <c r="E26" s="14"/>
       <c r="F26" s="14"/>
@@ -6942,18 +6942,18 @@
       <c r="H26" s="14"/>
       <c r="I26" s="14"/>
       <c r="J26" s="14"/>
-      <c r="K26" s="22"/>
+      <c r="K26" s="25"/>
       <c r="L26" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="16">
         <v>18</v>
       </c>
       <c r="B27" s="3"/>
-      <c r="C27" s="22"/>
+      <c r="C27" s="25"/>
       <c r="D27" s="14"/>
       <c r="E27" s="14"/>
       <c r="F27" s="14"/>
@@ -6961,18 +6961,18 @@
       <c r="H27" s="14"/>
       <c r="I27" s="14"/>
       <c r="J27" s="14"/>
-      <c r="K27" s="22"/>
+      <c r="K27" s="25"/>
       <c r="L27" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="16">
         <v>19</v>
       </c>
       <c r="B28" s="3"/>
-      <c r="C28" s="22"/>
+      <c r="C28" s="25"/>
       <c r="D28" s="14"/>
       <c r="E28" s="14"/>
       <c r="F28" s="14"/>
@@ -6980,18 +6980,18 @@
       <c r="H28" s="14"/>
       <c r="I28" s="14"/>
       <c r="J28" s="14"/>
-      <c r="K28" s="22"/>
+      <c r="K28" s="25"/>
       <c r="L28" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" s="16">
         <v>20</v>
       </c>
       <c r="B29" s="3"/>
-      <c r="C29" s="22"/>
+      <c r="C29" s="25"/>
       <c r="D29" s="14"/>
       <c r="E29" s="14"/>
       <c r="F29" s="14"/>
@@ -6999,18 +6999,18 @@
       <c r="H29" s="14"/>
       <c r="I29" s="14"/>
       <c r="J29" s="14"/>
-      <c r="K29" s="22"/>
+      <c r="K29" s="25"/>
       <c r="L29" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="16">
         <v>21</v>
       </c>
       <c r="B30" s="5"/>
-      <c r="C30" s="22"/>
+      <c r="C30" s="25"/>
       <c r="D30" s="14"/>
       <c r="E30" s="15"/>
       <c r="F30" s="15"/>
@@ -7018,7 +7018,7 @@
       <c r="H30" s="15"/>
       <c r="I30" s="15"/>
       <c r="J30" s="15"/>
-      <c r="K30" s="22"/>
+      <c r="K30" s="25"/>
       <c r="L30" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -7051,16 +7051,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.140625" customWidth="1"/>
-    <col min="2" max="2" width="44.42578125" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" style="2"/>
-    <col min="9" max="9" width="12.28515625" customWidth="1"/>
+    <col min="1" max="1" width="4.109375" customWidth="1"/>
+    <col min="2" max="2" width="44.44140625" customWidth="1"/>
+    <col min="5" max="5" width="11.44140625" style="2"/>
+    <col min="9" max="9" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B1" s="24"/>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B1" s="21"/>
       <c r="C1" s="33" t="s">
         <v>24</v>
       </c>
@@ -7071,8 +7071,8 @@
       <c r="H1" s="33"/>
       <c r="I1" s="33"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="24"/>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B2" s="21"/>
       <c r="C2" s="33"/>
       <c r="D2" s="33"/>
       <c r="E2" s="33"/>
@@ -7081,83 +7081,83 @@
       <c r="H2" s="33"/>
       <c r="I2" s="33"/>
     </row>
-    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="24"/>
-      <c r="C3" s="29" t="s">
+    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="21"/>
+      <c r="C3" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="24"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
-      <c r="G4" s="29"/>
-      <c r="H4" s="29"/>
-      <c r="I4" s="29"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="24"/>
-      <c r="C5" s="27" t="s">
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B4" s="21"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="28"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B5" s="21"/>
+      <c r="C5" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
       <c r="H5" s="8" t="s">
         <v>27</v>
       </c>
       <c r="I5" s="9"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B6" s="24"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="24"/>
-      <c r="C7" s="27" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B6" s="21"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="24"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B7" s="21"/>
+      <c r="C7" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="27"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B8" s="24"/>
-      <c r="C8" s="27" t="s">
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="24"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B8" s="21"/>
+      <c r="C8" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27" t="s">
+      <c r="D8" s="24"/>
+      <c r="E8" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27" t="s">
+      <c r="F8" s="24"/>
+      <c r="G8" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="H8" s="27"/>
+      <c r="H8" s="24"/>
       <c r="I8" s="10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>0</v>
       </c>
@@ -7186,7 +7186,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>1</v>
       </c>
@@ -7220,7 +7220,7 @@
         <v>3.0761904761904759</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>2</v>
       </c>
@@ -7254,7 +7254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>3</v>
       </c>
@@ -7288,7 +7288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>4</v>
       </c>
@@ -7322,7 +7322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>5</v>
       </c>
@@ -7356,7 +7356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>6</v>
       </c>
@@ -7390,7 +7390,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>7</v>
       </c>
@@ -7424,7 +7424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>8</v>
       </c>
@@ -7458,7 +7458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>9</v>
       </c>
@@ -7492,7 +7492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>10</v>
       </c>
@@ -7526,7 +7526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>11</v>
       </c>
@@ -7560,7 +7560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>12</v>
       </c>
@@ -7594,7 +7594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>13</v>
       </c>
@@ -7628,7 +7628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>14</v>
       </c>
@@ -7662,7 +7662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>15</v>
       </c>
@@ -7696,7 +7696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>16</v>
       </c>
@@ -7730,7 +7730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>17</v>
       </c>
@@ -7764,7 +7764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>18</v>
       </c>
@@ -7798,7 +7798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>19</v>
       </c>
@@ -7832,7 +7832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>20</v>
       </c>
@@ -7866,7 +7866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>21</v>
       </c>

</xml_diff>